<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-16 21:26 UTC
</commit_message>
<xml_diff>
--- a/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
+++ b/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
@@ -227,7 +227,7 @@
     <t>propuesta motor</t>
   </si>
   <si>
-    <t>Propuesta compras:,motor 4360</t>
+    <t>Propuesta compras:,motor ot 4360</t>
   </si>
   <si>
     <t>1215727723502427</t>
@@ -244,7 +244,7 @@
 </t>
   </si>
   <si>
-    <t>Propuesta compras:,Alabe 4360</t>
+    <t>Propuesta compras:,Alabe  ot 4360</t>
   </si>
   <si>
     <t>1215728035784425</t>
@@ -316,7 +316,7 @@
     <t>Reserva producción</t>
   </si>
   <si>
-    <t>motor 4360,Alabe 4360</t>
+    <t>motor ot 4360,Alabe  ot 4360</t>
   </si>
   <si>
     <t>Baja</t>
@@ -325,7 +325,7 @@
     <t>1215771707606683</t>
   </si>
   <si>
-    <t>motor 4360</t>
+    <t>motor ot 4360</t>
   </si>
   <si>
     <t>Reserva producción,Recepcionx motor</t>
@@ -334,7 +334,7 @@
     <t>1215771707606685</t>
   </si>
   <si>
-    <t>Alabe 4360</t>
+    <t>Alabe  ot 4360</t>
   </si>
   <si>
     <t>Reserva producción,Recepcionx Alabe</t>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="9">
-        <v>46189.81491765047</v>
+        <v>46189.89213912037</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>96</v>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46189.8148409375</v>
+        <v>46189.89217115741</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>99</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-19 17:06 Chile
</commit_message>
<xml_diff>
--- a/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
+++ b/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
@@ -1683,7 +1683,7 @@
         <v>46188.919674178236</v>
       </c>
       <c r="D5" s="9">
-        <v>46188.91968832176</v>
+        <v>46222.63597420139</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1748,7 +1748,7 @@
         <v>46188.919543298616</v>
       </c>
       <c r="D6" s="5">
-        <v>46213.76143587963</v>
+        <v>46222.635976273144</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>34</v>

</xml_diff>